<commit_message>
Mi primer commit desde la PC local
</commit_message>
<xml_diff>
--- a/Momento 1 Prueba de escritorio.xlsx
+++ b/Momento 1 Prueba de escritorio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Momento 1 LDP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DADBAE-5D65-46CA-8649-1A89A22FED69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF585041-2419-49A3-A113-EA0FB2F1C3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1BD7FB42-3E64-4BE2-8859-E1CF03D7BE8F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1BD7FB42-3E64-4BE2-8859-E1CF03D7BE8F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="48">
   <si>
     <t>InicioCosteoPrecios</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t>Variable de trabajo, Indica el valor de los impuestos (IVA) que se aplica al subtotal, tipo decimal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Arroz" </t>
   </si>
 </sst>
 </file>
@@ -202,16 +205,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -888,7 +890,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
         <v>37</v>
@@ -917,7 +919,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
         <v>37</v>
@@ -946,7 +948,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C15">
         <v>50000</v>
@@ -975,7 +977,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C16">
         <v>50000</v>
@@ -1004,7 +1006,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C17">
         <v>50000</v>
@@ -1030,7 +1032,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C18">
         <v>50000</v>
@@ -1059,7 +1061,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C19">
         <v>50000</v>
@@ -1088,7 +1090,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C20">
         <v>50000</v>
@@ -1117,7 +1119,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C21">
         <v>50000</v>
@@ -1146,7 +1148,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C22">
         <v>50000</v>
@@ -1175,7 +1177,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C23">
         <v>50000</v>
@@ -1204,7 +1206,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C24">
         <v>50000</v>
@@ -1233,7 +1235,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C25">
         <v>50000</v>
@@ -1262,7 +1264,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C26">
         <v>50000</v>
@@ -1291,7 +1293,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C27">
         <v>50000</v>
@@ -1320,7 +1322,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C28">
         <v>50000</v>
@@ -1349,7 +1351,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C29">
         <v>50000</v>
@@ -1375,7 +1377,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C30">
         <v>50000</v>
@@ -1404,7 +1406,7 @@
         <v>28</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C31">
         <v>50000</v>
@@ -1435,27 +1437,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3619111-590A-4CF7-AAB3-3C67242D2DD2}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1479,130 +1481,127 @@
       <c r="A3" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="K12" s="4"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>